<commit_message>
desestacionalizacion de mora total y mora de microcreditos
</commit_message>
<xml_diff>
--- a/outputs/datos_desestacionalizados.xlsx
+++ b/outputs/datos_desestacionalizados.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C253"/>
+  <dimension ref="A1:C219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,10 +454,10 @@
         <v>37288</v>
       </c>
       <c r="B3" t="n">
-        <v>0.07402339354629145</v>
+        <v>0.07432554810525711</v>
       </c>
       <c r="C3" t="n">
-        <v>0.05720757821436993</v>
+        <v>0.05739681144602771</v>
       </c>
     </row>
     <row r="4">
@@ -465,10 +465,10 @@
         <v>37316</v>
       </c>
       <c r="B4" t="n">
-        <v>0.07636255503576565</v>
+        <v>0.0770406299682367</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05923165593854857</v>
+        <v>0.05986908175523309</v>
       </c>
     </row>
     <row r="5">
@@ -476,10 +476,10 @@
         <v>37347</v>
       </c>
       <c r="B5" t="n">
-        <v>0.07392334804056314</v>
+        <v>0.07453901484739667</v>
       </c>
       <c r="C5" t="n">
-        <v>0.05690251778802776</v>
+        <v>0.05749019747812037</v>
       </c>
     </row>
     <row r="6">
@@ -487,10 +487,10 @@
         <v>37377</v>
       </c>
       <c r="B6" t="n">
-        <v>0.0722185575984689</v>
+        <v>0.0727176921834905</v>
       </c>
       <c r="C6" t="n">
-        <v>0.05584307338801648</v>
+        <v>0.05637696414471354</v>
       </c>
     </row>
     <row r="7">
@@ -498,10 +498,10 @@
         <v>37408</v>
       </c>
       <c r="B7" t="n">
-        <v>0.07227346117146835</v>
+        <v>0.0726906979430577</v>
       </c>
       <c r="C7" t="n">
-        <v>0.05535203454979339</v>
+        <v>0.05584840006394314</v>
       </c>
     </row>
     <row r="8">
@@ -509,10 +509,10 @@
         <v>37438</v>
       </c>
       <c r="B8" t="n">
-        <v>0.06805310470469927</v>
+        <v>0.06824222611814519</v>
       </c>
       <c r="C8" t="n">
-        <v>0.05288049940759765</v>
+        <v>0.05323761549150356</v>
       </c>
     </row>
     <row r="9">
@@ -520,10 +520,10 @@
         <v>37469</v>
       </c>
       <c r="B9" t="n">
-        <v>0.06481475128586141</v>
+        <v>0.0647666482851967</v>
       </c>
       <c r="C9" t="n">
-        <v>0.04962981205432671</v>
+        <v>0.04978012248045369</v>
       </c>
     </row>
     <row r="10">
@@ -531,10 +531,10 @@
         <v>37500</v>
       </c>
       <c r="B10" t="n">
-        <v>0.06418052939067856</v>
+        <v>0.06410722682985288</v>
       </c>
       <c r="C10" t="n">
-        <v>0.04884474711343995</v>
+        <v>0.04901363925234872</v>
       </c>
     </row>
     <row r="11">
@@ -542,10 +542,10 @@
         <v>37530</v>
       </c>
       <c r="B11" t="n">
-        <v>0.06402535870230765</v>
+        <v>0.06388477439078094</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0465370778272553</v>
+        <v>0.04665695766451193</v>
       </c>
     </row>
     <row r="12">
@@ -553,10 +553,10 @@
         <v>37561</v>
       </c>
       <c r="B12" t="n">
-        <v>0.0632713078144987</v>
+        <v>0.06335634430244262</v>
       </c>
       <c r="C12" t="n">
-        <v>0.046557953971036</v>
+        <v>0.04675236788157629</v>
       </c>
     </row>
     <row r="13">
@@ -564,10 +564,10 @@
         <v>37591</v>
       </c>
       <c r="B13" t="n">
-        <v>0.06324536372576099</v>
+        <v>0.06338334436650155</v>
       </c>
       <c r="C13" t="n">
-        <v>0.04692357022318815</v>
+        <v>0.04705565191908068</v>
       </c>
     </row>
     <row r="14">
@@ -586,10 +586,10 @@
         <v>37653</v>
       </c>
       <c r="B15" t="n">
-        <v>0.06070743570232991</v>
+        <v>0.06100959026129557</v>
       </c>
       <c r="C15" t="n">
-        <v>0.04483285649625397</v>
+        <v>0.04502208972791175</v>
       </c>
     </row>
     <row r="16">
@@ -597,10 +597,10 @@
         <v>37681</v>
       </c>
       <c r="B16" t="n">
-        <v>0.06255695765036536</v>
+        <v>0.0632350325828364</v>
       </c>
       <c r="C16" t="n">
-        <v>0.04607376570427236</v>
+        <v>0.04671119152095687</v>
       </c>
     </row>
     <row r="17">
@@ -608,10 +608,10 @@
         <v>37712</v>
       </c>
       <c r="B17" t="n">
-        <v>0.06261713904951789</v>
+        <v>0.06323280585635142</v>
       </c>
       <c r="C17" t="n">
-        <v>0.046243335815671</v>
+        <v>0.04683101550576361</v>
       </c>
     </row>
     <row r="18">
@@ -619,10 +619,10 @@
         <v>37742</v>
       </c>
       <c r="B18" t="n">
-        <v>0.06308396204687006</v>
+        <v>0.06358309663189166</v>
       </c>
       <c r="C18" t="n">
-        <v>0.04675678413837362</v>
+        <v>0.04729067489507068</v>
       </c>
     </row>
     <row r="19">
@@ -630,10 +630,10 @@
         <v>37773</v>
       </c>
       <c r="B19" t="n">
-        <v>0.06431197491881131</v>
+        <v>0.06472921169040066</v>
       </c>
       <c r="C19" t="n">
-        <v>0.04852723410659176</v>
+        <v>0.04902359962074151</v>
       </c>
     </row>
     <row r="20">
@@ -641,10 +641,10 @@
         <v>37803</v>
       </c>
       <c r="B20" t="n">
-        <v>0.06281618567969489</v>
+        <v>0.06300530709314081</v>
       </c>
       <c r="C20" t="n">
-        <v>0.04707077394961878</v>
+        <v>0.04742789003352468</v>
       </c>
     </row>
     <row r="21">
@@ -652,10 +652,10 @@
         <v>37834</v>
       </c>
       <c r="B21" t="n">
-        <v>0.06424255422554739</v>
+        <v>0.06419445122488268</v>
       </c>
       <c r="C21" t="n">
-        <v>0.04800848598583503</v>
+        <v>0.04815879641196201</v>
       </c>
     </row>
     <row r="22">
@@ -663,10 +663,10 @@
         <v>37865</v>
       </c>
       <c r="B22" t="n">
-        <v>0.0666328515277943</v>
+        <v>0.06655954896696863</v>
       </c>
       <c r="C22" t="n">
-        <v>0.04927905197987626</v>
+        <v>0.04944794411878504</v>
       </c>
     </row>
     <row r="23">
@@ -674,10 +674,10 @@
         <v>37895</v>
       </c>
       <c r="B23" t="n">
-        <v>0.06413491427800956</v>
+        <v>0.06399432996648285</v>
       </c>
       <c r="C23" t="n">
-        <v>0.04818015636065958</v>
+        <v>0.04830003619791622</v>
       </c>
     </row>
     <row r="24">
@@ -685,10 +685,10 @@
         <v>37926</v>
       </c>
       <c r="B24" t="n">
-        <v>0.06224973611377058</v>
+        <v>0.06233477260171449</v>
       </c>
       <c r="C24" t="n">
-        <v>0.04805793478112844</v>
+        <v>0.04825234869166873</v>
       </c>
     </row>
     <row r="25">
@@ -696,10 +696,10 @@
         <v>37956</v>
       </c>
       <c r="B25" t="n">
-        <v>0.0640474992610833</v>
+        <v>0.06418547990182386</v>
       </c>
       <c r="C25" t="n">
-        <v>0.04884892167532816</v>
+        <v>0.04898100337122069</v>
       </c>
     </row>
     <row r="26">
@@ -718,10 +718,10 @@
         <v>38018</v>
       </c>
       <c r="B27" t="n">
-        <v>0.06492505956136756</v>
+        <v>0.06522721412033322</v>
       </c>
       <c r="C27" t="n">
-        <v>0.04866174505017896</v>
+        <v>0.04885097828183675</v>
       </c>
     </row>
     <row r="28">
@@ -729,10 +729,10 @@
         <v>38047</v>
       </c>
       <c r="B28" t="n">
-        <v>0.06551024412687378</v>
+        <v>0.06618831905934483</v>
       </c>
       <c r="C28" t="n">
-        <v>0.04912979126155594</v>
+        <v>0.04976721707824046</v>
       </c>
     </row>
     <row r="29">
@@ -740,10 +740,10 @@
         <v>38078</v>
       </c>
       <c r="B29" t="n">
-        <v>0.06697017843166929</v>
+        <v>0.06758584523850282</v>
       </c>
       <c r="C29" t="n">
-        <v>0.04972872566219555</v>
+        <v>0.05031640535228816</v>
       </c>
     </row>
     <row r="30">
@@ -751,10 +751,10 @@
         <v>38108</v>
       </c>
       <c r="B30" t="n">
-        <v>0.06617392280524248</v>
+        <v>0.06667305739026408</v>
       </c>
       <c r="C30" t="n">
-        <v>0.05008757863293715</v>
+        <v>0.05062146938963421</v>
       </c>
     </row>
     <row r="31">
@@ -762,10 +762,10 @@
         <v>38139</v>
       </c>
       <c r="B31" t="n">
-        <v>0.07291637577434293</v>
+        <v>0.07333361254593228</v>
       </c>
       <c r="C31" t="n">
-        <v>0.05431945487543931</v>
+        <v>0.05481582038958906</v>
       </c>
     </row>
     <row r="32">
@@ -773,10 +773,10 @@
         <v>38169</v>
       </c>
       <c r="B32" t="n">
-        <v>0.07493329443815813</v>
+        <v>0.07512241585160405</v>
       </c>
       <c r="C32" t="n">
-        <v>0.0559860530697202</v>
+        <v>0.0563431691536261</v>
       </c>
     </row>
     <row r="33">
@@ -784,10 +784,10 @@
         <v>38200</v>
       </c>
       <c r="B33" t="n">
-        <v>0.07400239485538591</v>
+        <v>0.0739542918547212</v>
       </c>
       <c r="C33" t="n">
-        <v>0.05562807294807152</v>
+        <v>0.05577838337419851</v>
       </c>
     </row>
     <row r="34">
@@ -795,10 +795,10 @@
         <v>38231</v>
       </c>
       <c r="B34" t="n">
-        <v>0.07206542560879044</v>
+        <v>0.07199212304796476</v>
       </c>
       <c r="C34" t="n">
-        <v>0.05422940022056233</v>
+        <v>0.05439829235947111</v>
       </c>
     </row>
     <row r="35">
@@ -806,10 +806,10 @@
         <v>38261</v>
       </c>
       <c r="B35" t="n">
-        <v>0.06962917987690204</v>
+        <v>0.06948859556537533</v>
       </c>
       <c r="C35" t="n">
-        <v>0.05350387081886379</v>
+        <v>0.05362375065612043</v>
       </c>
     </row>
     <row r="36">
@@ -817,10 +817,10 @@
         <v>38292</v>
       </c>
       <c r="B36" t="n">
-        <v>0.06921539336875294</v>
+        <v>0.06930042985669686</v>
       </c>
       <c r="C36" t="n">
-        <v>0.05255534302115583</v>
+        <v>0.05274975693169612</v>
       </c>
     </row>
     <row r="37">
@@ -828,10 +828,10 @@
         <v>38322</v>
       </c>
       <c r="B37" t="n">
-        <v>0.07430649442643825</v>
+        <v>0.0744444750671788</v>
       </c>
       <c r="C37" t="n">
-        <v>0.0555040153267216</v>
+        <v>0.05563609702261412</v>
       </c>
     </row>
     <row r="38">
@@ -850,10 +850,10 @@
         <v>38384</v>
       </c>
       <c r="B39" t="n">
-        <v>0.07763838935023182</v>
+        <v>0.07794054390919748</v>
       </c>
       <c r="C39" t="n">
-        <v>0.05706515216142569</v>
+        <v>0.05725438539308348</v>
       </c>
     </row>
     <row r="40">
@@ -861,10 +861,10 @@
         <v>38412</v>
       </c>
       <c r="B40" t="n">
-        <v>0.07691153744499735</v>
+        <v>0.07758961237746839</v>
       </c>
       <c r="C40" t="n">
-        <v>0.05608384550093309</v>
+        <v>0.05672127131761761</v>
       </c>
     </row>
     <row r="41">
@@ -872,10 +872,10 @@
         <v>38443</v>
       </c>
       <c r="B41" t="n">
-        <v>0.07629693874511073</v>
+        <v>0.07691260555194426</v>
       </c>
       <c r="C41" t="n">
-        <v>0.05536515609713967</v>
+        <v>0.05595283578723228</v>
       </c>
     </row>
     <row r="42">
@@ -883,10 +883,10 @@
         <v>38473</v>
       </c>
       <c r="B42" t="n">
-        <v>0.07656146053896033</v>
+        <v>0.07706059512398193</v>
       </c>
       <c r="C42" t="n">
-        <v>0.05561651904228247</v>
+        <v>0.05615040979897953</v>
       </c>
     </row>
     <row r="43">
@@ -894,10 +894,10 @@
         <v>38504</v>
       </c>
       <c r="B43" t="n">
-        <v>0.07471827048284045</v>
+        <v>0.0751355072544298</v>
       </c>
       <c r="C43" t="n">
-        <v>0.05431352195364776</v>
+        <v>0.05480988746779751</v>
       </c>
     </row>
     <row r="44">
@@ -905,10 +905,10 @@
         <v>38534</v>
       </c>
       <c r="B44" t="n">
-        <v>0.07593938539994574</v>
+        <v>0.07612850681339166</v>
       </c>
       <c r="C44" t="n">
-        <v>0.05430612097663975</v>
+        <v>0.05466323706054566</v>
       </c>
     </row>
     <row r="45">
@@ -916,10 +916,10 @@
         <v>38565</v>
       </c>
       <c r="B45" t="n">
-        <v>0.07313187184457499</v>
+        <v>0.07308376884391028</v>
       </c>
       <c r="C45" t="n">
-        <v>0.05305908199506365</v>
+        <v>0.05320939242119063</v>
       </c>
     </row>
     <row r="46">
@@ -927,10 +927,10 @@
         <v>38596</v>
       </c>
       <c r="B46" t="n">
-        <v>0.07306774092952499</v>
+        <v>0.07299443836869932</v>
       </c>
       <c r="C46" t="n">
-        <v>0.05343138811015292</v>
+        <v>0.0536002802490617</v>
       </c>
     </row>
     <row r="47">
@@ -938,10 +938,10 @@
         <v>38626</v>
       </c>
       <c r="B47" t="n">
-        <v>0.07238132519542194</v>
+        <v>0.07224074088389523</v>
       </c>
       <c r="C47" t="n">
-        <v>0.05328514467988845</v>
+        <v>0.05340502451714509</v>
       </c>
     </row>
     <row r="48">
@@ -949,10 +949,10 @@
         <v>38657</v>
       </c>
       <c r="B48" t="n">
-        <v>0.06965512093366096</v>
+        <v>0.06974015742160487</v>
       </c>
       <c r="C48" t="n">
-        <v>0.05115352243821961</v>
+        <v>0.05134793634875991</v>
       </c>
     </row>
     <row r="49">
@@ -960,10 +960,10 @@
         <v>38687</v>
       </c>
       <c r="B49" t="n">
-        <v>0.06821390851113274</v>
+        <v>0.0683518891518733</v>
       </c>
       <c r="C49" t="n">
-        <v>0.05177630019811477</v>
+        <v>0.0519083818940073</v>
       </c>
     </row>
     <row r="50">
@@ -982,10 +982,10 @@
         <v>38749</v>
       </c>
       <c r="B51" t="n">
-        <v>0.06797949856993631</v>
+        <v>0.06828165312890197</v>
       </c>
       <c r="C51" t="n">
-        <v>0.05154871847128092</v>
+        <v>0.0517379517029387</v>
       </c>
     </row>
     <row r="52">
@@ -993,10 +993,10 @@
         <v>38777</v>
       </c>
       <c r="B52" t="n">
-        <v>0.06589454878470695</v>
+        <v>0.06657262371717799</v>
       </c>
       <c r="C52" t="n">
-        <v>0.05037585607873973</v>
+        <v>0.05101328189542425</v>
       </c>
     </row>
     <row r="53">
@@ -1004,10 +1004,10 @@
         <v>38808</v>
       </c>
       <c r="B53" t="n">
-        <v>0.06489777302387806</v>
+        <v>0.06551343983071159</v>
       </c>
       <c r="C53" t="n">
-        <v>0.05093715242781544</v>
+        <v>0.05152483211790804</v>
       </c>
     </row>
     <row r="54">
@@ -1015,10 +1015,10 @@
         <v>38838</v>
       </c>
       <c r="B54" t="n">
-        <v>0.06477951415519649</v>
+        <v>0.06527864874021809</v>
       </c>
       <c r="C54" t="n">
-        <v>0.05014969082844295</v>
+        <v>0.05068358158514001</v>
       </c>
     </row>
     <row r="55">
@@ -1026,10 +1026,10 @@
         <v>38869</v>
       </c>
       <c r="B55" t="n">
-        <v>0.06591753243437072</v>
+        <v>0.06633476920596007</v>
       </c>
       <c r="C55" t="n">
-        <v>0.05092182352291979</v>
+        <v>0.05141818903706954</v>
       </c>
     </row>
     <row r="56">
@@ -1037,10 +1037,10 @@
         <v>38899</v>
       </c>
       <c r="B56" t="n">
-        <v>0.06580707044967059</v>
+        <v>0.0659961918631165</v>
       </c>
       <c r="C56" t="n">
-        <v>0.05068024990034348</v>
+        <v>0.05103736598424938</v>
       </c>
     </row>
     <row r="57">
@@ -1048,10 +1048,10 @@
         <v>38930</v>
       </c>
       <c r="B57" t="n">
-        <v>0.065686320169563</v>
+        <v>0.06563821716889828</v>
       </c>
       <c r="C57" t="n">
-        <v>0.05033903837760708</v>
+        <v>0.05048934880373406</v>
       </c>
     </row>
     <row r="58">
@@ -1059,10 +1059,10 @@
         <v>38961</v>
       </c>
       <c r="B58" t="n">
-        <v>0.06658239838059994</v>
+        <v>0.06650909581977427</v>
       </c>
       <c r="C58" t="n">
-        <v>0.05016665783946556</v>
+        <v>0.05033554997837433</v>
       </c>
     </row>
     <row r="59">
@@ -1070,10 +1070,10 @@
         <v>38991</v>
       </c>
       <c r="B59" t="n">
-        <v>0.06678190031372756</v>
+        <v>0.06664131600220086</v>
       </c>
       <c r="C59" t="n">
-        <v>0.05069220713574371</v>
+        <v>0.05081208697300035</v>
       </c>
     </row>
     <row r="60">
@@ -1081,10 +1081,10 @@
         <v>39022</v>
       </c>
       <c r="B60" t="n">
-        <v>0.06468420252460684</v>
+        <v>0.06476923901255076</v>
       </c>
       <c r="C60" t="n">
-        <v>0.04998423555657428</v>
+        <v>0.05017864946711457</v>
       </c>
     </row>
     <row r="61">
@@ -1092,10 +1092,10 @@
         <v>39052</v>
       </c>
       <c r="B61" t="n">
-        <v>0.06398445487651061</v>
+        <v>0.06412243551725116</v>
       </c>
       <c r="C61" t="n">
-        <v>0.04863896528715694</v>
+        <v>0.04877104698304947</v>
       </c>
     </row>
     <row r="62">
@@ -1114,10 +1114,10 @@
         <v>39114</v>
       </c>
       <c r="B63" t="n">
-        <v>0.06522025599856322</v>
+        <v>0.06552241055752889</v>
       </c>
       <c r="C63" t="n">
-        <v>0.04794823166789954</v>
+        <v>0.04813746489955732</v>
       </c>
     </row>
     <row r="64">
@@ -1125,10 +1125,10 @@
         <v>39142</v>
       </c>
       <c r="B64" t="n">
-        <v>0.06379219914470778</v>
+        <v>0.06447027407717883</v>
       </c>
       <c r="C64" t="n">
-        <v>0.04707729474518552</v>
+        <v>0.04771472056187004</v>
       </c>
     </row>
     <row r="65">
@@ -1136,10 +1136,10 @@
         <v>39173</v>
       </c>
       <c r="B65" t="n">
-        <v>0.06343482097958679</v>
+        <v>0.06405048778642032</v>
       </c>
       <c r="C65" t="n">
-        <v>0.04663094824393837</v>
+        <v>0.04721862793403098</v>
       </c>
     </row>
     <row r="66">
@@ -1147,10 +1147,10 @@
         <v>39203</v>
       </c>
       <c r="B66" t="n">
-        <v>0.06250879670490093</v>
+        <v>0.06300793128992253</v>
       </c>
       <c r="C66" t="n">
-        <v>0.04548018791827257</v>
+        <v>0.04601407867496964</v>
       </c>
     </row>
     <row r="67">
@@ -1158,10 +1158,10 @@
         <v>39234</v>
       </c>
       <c r="B67" t="n">
-        <v>0.06132096744016043</v>
+        <v>0.06173820421174978</v>
       </c>
       <c r="C67" t="n">
-        <v>0.04454401782905744</v>
+        <v>0.04504038334320719</v>
       </c>
     </row>
     <row r="68">
@@ -1169,10 +1169,10 @@
         <v>39264</v>
       </c>
       <c r="B68" t="n">
-        <v>0.05988641701661269</v>
+        <v>0.06007553843005861</v>
       </c>
       <c r="C68" t="n">
-        <v>0.04295300815717402</v>
+        <v>0.04331012424107993</v>
       </c>
     </row>
     <row r="69">
@@ -1180,10 +1180,10 @@
         <v>39295</v>
       </c>
       <c r="B69" t="n">
-        <v>0.05998657046991633</v>
+        <v>0.05993846746925163</v>
       </c>
       <c r="C69" t="n">
-        <v>0.04363853668449275</v>
+        <v>0.04378884711061973</v>
       </c>
     </row>
     <row r="70">
@@ -1191,10 +1191,10 @@
         <v>39326</v>
       </c>
       <c r="B70" t="n">
-        <v>0.05986648522527754</v>
+        <v>0.05979318266445187</v>
       </c>
       <c r="C70" t="n">
-        <v>0.04378104819033531</v>
+        <v>0.04394994032924408</v>
       </c>
     </row>
     <row r="71">
@@ -1202,10 +1202,10 @@
         <v>39356</v>
       </c>
       <c r="B71" t="n">
-        <v>0.05906355655465776</v>
+        <v>0.05892297224313105</v>
       </c>
       <c r="C71" t="n">
-        <v>0.04304792436436861</v>
+        <v>0.04316780420162524</v>
       </c>
     </row>
     <row r="72">
@@ -1213,10 +1213,10 @@
         <v>39387</v>
       </c>
       <c r="B72" t="n">
-        <v>0.05636916712360798</v>
+        <v>0.05645420361155189</v>
       </c>
       <c r="C72" t="n">
-        <v>0.04178275543382372</v>
+        <v>0.04197716934436402</v>
       </c>
     </row>
     <row r="73">
@@ -1224,10 +1224,10 @@
         <v>39417</v>
       </c>
       <c r="B73" t="n">
-        <v>0.05796694949119499</v>
+        <v>0.05810493013193555</v>
       </c>
       <c r="C73" t="n">
-        <v>0.04310961056784608</v>
+        <v>0.0432416922637386</v>
       </c>
     </row>
     <row r="74">
@@ -1246,10 +1246,10 @@
         <v>39479</v>
       </c>
       <c r="B75" t="n">
-        <v>0.05499435078145719</v>
+        <v>0.05529650534042285</v>
       </c>
       <c r="C75" t="n">
-        <v>0.04046354294299023</v>
+        <v>0.04065277617464802</v>
       </c>
     </row>
     <row r="76">
@@ -1257,10 +1257,10 @@
         <v>39508</v>
       </c>
       <c r="B76" t="n">
-        <v>0.05753274522410456</v>
+        <v>0.05821082015657561</v>
       </c>
       <c r="C76" t="n">
-        <v>0.043602889657119</v>
+        <v>0.04424031547380352</v>
       </c>
     </row>
     <row r="77">
@@ -1268,10 +1268,10 @@
         <v>39539</v>
       </c>
       <c r="B77" t="n">
-        <v>0.05378740882065643</v>
+        <v>0.05440307562748996</v>
       </c>
       <c r="C77" t="n">
-        <v>0.04115649768495519</v>
+        <v>0.0417441773750478</v>
       </c>
     </row>
     <row r="78">
@@ -1279,10 +1279,10 @@
         <v>39569</v>
       </c>
       <c r="B78" t="n">
-        <v>0.05325764235199224</v>
+        <v>0.05375677693701384</v>
       </c>
       <c r="C78" t="n">
-        <v>0.04115726855967788</v>
+        <v>0.04169115931637495</v>
       </c>
     </row>
     <row r="79">
@@ -1290,10 +1290,10 @@
         <v>39600</v>
       </c>
       <c r="B79" t="n">
-        <v>0.05250930613699866</v>
+        <v>0.05292654290858801</v>
       </c>
       <c r="C79" t="n">
-        <v>0.04109303025406158</v>
+        <v>0.04158939576821133</v>
       </c>
     </row>
     <row r="80">
@@ -1301,10 +1301,10 @@
         <v>39630</v>
       </c>
       <c r="B80" t="n">
-        <v>0.05268756083008068</v>
+        <v>0.0528766822435266</v>
       </c>
       <c r="C80" t="n">
-        <v>0.04074263808241522</v>
+        <v>0.04109975416632113</v>
       </c>
     </row>
     <row r="81">
@@ -1312,10 +1312,10 @@
         <v>39661</v>
       </c>
       <c r="B81" t="n">
-        <v>0.05090135010890207</v>
+        <v>0.05085324710823737</v>
       </c>
       <c r="C81" t="n">
-        <v>0.03932954407782665</v>
+        <v>0.03947985450395363</v>
       </c>
     </row>
     <row r="82">
@@ -1323,10 +1323,10 @@
         <v>39692</v>
       </c>
       <c r="B82" t="n">
-        <v>0.05066238930718454</v>
+        <v>0.05058908674635887</v>
       </c>
       <c r="C82" t="n">
-        <v>0.0397656781695483</v>
+        <v>0.03993457030845708</v>
       </c>
     </row>
     <row r="83">
@@ -1334,10 +1334,10 @@
         <v>39722</v>
       </c>
       <c r="B83" t="n">
-        <v>0.05079434493032878</v>
+        <v>0.05065376061880208</v>
       </c>
       <c r="C83" t="n">
-        <v>0.04005778536818332</v>
+        <v>0.04017766520543996</v>
       </c>
     </row>
     <row r="84">
@@ -1345,10 +1345,10 @@
         <v>39753</v>
       </c>
       <c r="B84" t="n">
-        <v>0.0528315001334636</v>
+        <v>0.05291653662140752</v>
       </c>
       <c r="C84" t="n">
-        <v>0.0416469701436657</v>
+        <v>0.04184138405420599</v>
       </c>
     </row>
     <row r="85">
@@ -1356,10 +1356,10 @@
         <v>39783</v>
       </c>
       <c r="B85" t="n">
-        <v>0.05386163803884276</v>
+        <v>0.05399961867958332</v>
       </c>
       <c r="C85" t="n">
-        <v>0.04379663824360611</v>
+        <v>0.04392871993949864</v>
       </c>
     </row>
     <row r="86">
@@ -1378,10 +1378,10 @@
         <v>39845</v>
       </c>
       <c r="B87" t="n">
-        <v>0.05214252029215852</v>
+        <v>0.05244467485112418</v>
       </c>
       <c r="C87" t="n">
-        <v>0.04366419769238881</v>
+        <v>0.0438534309240466</v>
       </c>
     </row>
     <row r="88">
@@ -1389,10 +1389,10 @@
         <v>39873</v>
       </c>
       <c r="B88" t="n">
-        <v>0.05195541690732654</v>
+        <v>0.05263349183979759</v>
       </c>
       <c r="C88" t="n">
-        <v>0.04275610154245771</v>
+        <v>0.04339352735914222</v>
       </c>
     </row>
     <row r="89">
@@ -1400,10 +1400,10 @@
         <v>39904</v>
       </c>
       <c r="B89" t="n">
-        <v>0.05291041234818614</v>
+        <v>0.05352607915501967</v>
       </c>
       <c r="C89" t="n">
-        <v>0.04385491378581005</v>
+        <v>0.04444259347590266</v>
       </c>
     </row>
     <row r="90">
@@ -1411,10 +1411,10 @@
         <v>39934</v>
       </c>
       <c r="B90" t="n">
-        <v>0.05374904973137732</v>
+        <v>0.05424818431639892</v>
       </c>
       <c r="C90" t="n">
-        <v>0.04432534317042016</v>
+        <v>0.04485923392711722</v>
       </c>
     </row>
     <row r="91">
@@ -1422,10 +1422,10 @@
         <v>39965</v>
       </c>
       <c r="B91" t="n">
-        <v>0.05674521096341429</v>
+        <v>0.05716244773500364</v>
       </c>
       <c r="C91" t="n">
-        <v>0.04734890398759671</v>
+        <v>0.04784526950174646</v>
       </c>
     </row>
     <row r="92">
@@ -1433,10 +1433,10 @@
         <v>39995</v>
       </c>
       <c r="B92" t="n">
-        <v>0.05815284729406427</v>
+        <v>0.05834196870751018</v>
       </c>
       <c r="C92" t="n">
-        <v>0.04849421448975189</v>
+        <v>0.0488513305736578</v>
       </c>
     </row>
     <row r="93">
@@ -1444,10 +1444,10 @@
         <v>40026</v>
       </c>
       <c r="B93" t="n">
-        <v>0.05910003357417024</v>
+        <v>0.05905193057350554</v>
       </c>
       <c r="C93" t="n">
-        <v>0.0487622493814696</v>
+        <v>0.04891255980759658</v>
       </c>
     </row>
     <row r="94">
@@ -1455,10 +1455,10 @@
         <v>40057</v>
       </c>
       <c r="B94" t="n">
-        <v>0.06062614797983449</v>
+        <v>0.06055284541900881</v>
       </c>
       <c r="C94" t="n">
-        <v>0.04996112436208605</v>
+        <v>0.05013001650099483</v>
       </c>
     </row>
     <row r="95">
@@ -1466,10 +1466,10 @@
         <v>40087</v>
       </c>
       <c r="B95" t="n">
-        <v>0.06317022243229785</v>
+        <v>0.06302963812077114</v>
       </c>
       <c r="C95" t="n">
-        <v>0.05156444862405096</v>
+        <v>0.05168432846130759</v>
       </c>
     </row>
     <row r="96">
@@ -1477,10 +1477,10 @@
         <v>40118</v>
       </c>
       <c r="B96" t="n">
-        <v>0.06664310348741373</v>
+        <v>0.06672813997535765</v>
       </c>
       <c r="C96" t="n">
-        <v>0.05531169677875902</v>
+        <v>0.05550611068929931</v>
       </c>
     </row>
     <row r="97">
@@ -1488,10 +1488,10 @@
         <v>40148</v>
       </c>
       <c r="B97" t="n">
-        <v>0.06785457768669925</v>
+        <v>0.06799255832743981</v>
       </c>
       <c r="C97" t="n">
-        <v>0.0560113052067143</v>
+        <v>0.05614338690260683</v>
       </c>
     </row>
     <row r="98">
@@ -1510,10 +1510,10 @@
         <v>40210</v>
       </c>
       <c r="B99" t="n">
-        <v>0.07079943663505452</v>
+        <v>0.07110159119402018</v>
       </c>
       <c r="C99" t="n">
-        <v>0.05993026060131468</v>
+        <v>0.06011949383297246</v>
       </c>
     </row>
     <row r="100">
@@ -1521,10 +1521,10 @@
         <v>40238</v>
       </c>
       <c r="B100" t="n">
-        <v>0.06974944508141896</v>
+        <v>0.07042752001389001</v>
       </c>
       <c r="C100" t="n">
-        <v>0.05876777437924554</v>
+        <v>0.05940520019593006</v>
       </c>
     </row>
     <row r="101">
@@ -1532,10 +1532,10 @@
         <v>40269</v>
       </c>
       <c r="B101" t="n">
-        <v>0.07147148175025131</v>
+        <v>0.07208714855708484</v>
       </c>
       <c r="C101" t="n">
-        <v>0.05959208168860995</v>
+        <v>0.06017976137870256</v>
       </c>
     </row>
     <row r="102">
@@ -1543,10 +1543,10 @@
         <v>40299</v>
       </c>
       <c r="B102" t="n">
-        <v>0.07234625181544996</v>
+        <v>0.07284538640047156</v>
       </c>
       <c r="C102" t="n">
-        <v>0.06002436670996581</v>
+        <v>0.06055825746666287</v>
       </c>
     </row>
     <row r="103">
@@ -1554,10 +1554,10 @@
         <v>40330</v>
       </c>
       <c r="B103" t="n">
-        <v>0.07465490703561468</v>
+        <v>0.07507214380720403</v>
       </c>
       <c r="C103" t="n">
-        <v>0.061631735534879</v>
+        <v>0.06212810104902874</v>
       </c>
     </row>
     <row r="104">
@@ -1565,10 +1565,10 @@
         <v>40360</v>
       </c>
       <c r="B104" t="n">
-        <v>0.07456634156894341</v>
+        <v>0.07475546298238933</v>
       </c>
       <c r="C104" t="n">
-        <v>0.06181822220546508</v>
+        <v>0.06217533828937099</v>
       </c>
     </row>
     <row r="105">
@@ -1576,10 +1576,10 @@
         <v>40391</v>
       </c>
       <c r="B105" t="n">
-        <v>0.07335127061050194</v>
+        <v>0.07330316760983722</v>
       </c>
       <c r="C105" t="n">
-        <v>0.06157156638623316</v>
+        <v>0.06172187681236014</v>
       </c>
     </row>
     <row r="106">
@@ -1587,10 +1587,10 @@
         <v>40422</v>
       </c>
       <c r="B106" t="n">
-        <v>0.0707799038555498</v>
+        <v>0.07070660129472413</v>
       </c>
       <c r="C106" t="n">
-        <v>0.05995869818872779</v>
+        <v>0.06012759032763657</v>
       </c>
     </row>
     <row r="107">
@@ -1598,10 +1598,10 @@
         <v>40452</v>
       </c>
       <c r="B107" t="n">
-        <v>0.07016552572568063</v>
+        <v>0.07002494141415393</v>
       </c>
       <c r="C107" t="n">
-        <v>0.05993610683080042</v>
+        <v>0.06005598666805706</v>
       </c>
     </row>
     <row r="108">
@@ -1609,10 +1609,10 @@
         <v>40483</v>
       </c>
       <c r="B108" t="n">
-        <v>0.06806771159863939</v>
+        <v>0.06815274808658331</v>
       </c>
       <c r="C108" t="n">
-        <v>0.05861590068014559</v>
+        <v>0.05881031459068588</v>
       </c>
     </row>
     <row r="109">
@@ -1620,10 +1620,10 @@
         <v>40513</v>
       </c>
       <c r="B109" t="n">
-        <v>0.06830768569903804</v>
+        <v>0.0684456663397786</v>
       </c>
       <c r="C109" t="n">
-        <v>0.05828031035483097</v>
+        <v>0.0584123920507235</v>
       </c>
     </row>
     <row r="110">
@@ -1642,10 +1642,10 @@
         <v>40575</v>
       </c>
       <c r="B111" t="n">
-        <v>0.06527674503370699</v>
+        <v>0.06557889959267266</v>
       </c>
       <c r="C111" t="n">
-        <v>0.05552534339076581</v>
+        <v>0.05571457662242359</v>
       </c>
     </row>
     <row r="112">
@@ -1653,10 +1653,10 @@
         <v>40603</v>
       </c>
       <c r="B112" t="n">
-        <v>0.06186647398770562</v>
+        <v>0.06254454892017666</v>
       </c>
       <c r="C112" t="n">
-        <v>0.05220357785208031</v>
+        <v>0.05284100366876483</v>
       </c>
     </row>
     <row r="113">
@@ -1664,10 +1664,10 @@
         <v>40634</v>
       </c>
       <c r="B113" t="n">
-        <v>0.06243065742338472</v>
+        <v>0.06304632423021825</v>
       </c>
       <c r="C113" t="n">
-        <v>0.05243324462999766</v>
+        <v>0.05302092432009026</v>
       </c>
     </row>
     <row r="114">
@@ -1675,10 +1675,10 @@
         <v>40664</v>
       </c>
       <c r="B114" t="n">
-        <v>0.06325683695966054</v>
+        <v>0.06375597154468214</v>
       </c>
       <c r="C114" t="n">
-        <v>0.05275587966145639</v>
+        <v>0.05328977041815345</v>
       </c>
     </row>
     <row r="115">
@@ -1686,10 +1686,10 @@
         <v>40695</v>
       </c>
       <c r="B115" t="n">
-        <v>0.062503256104319</v>
+        <v>0.06292049287590835</v>
       </c>
       <c r="C115" t="n">
-        <v>0.05232546074237126</v>
+        <v>0.05282182625652101</v>
       </c>
     </row>
     <row r="116">
@@ -1697,10 +1697,10 @@
         <v>40725</v>
       </c>
       <c r="B116" t="n">
-        <v>0.06484179433679077</v>
+        <v>0.06503091575023669</v>
       </c>
       <c r="C116" t="n">
-        <v>0.05391597324309654</v>
+        <v>0.05427308932700245</v>
       </c>
     </row>
     <row r="117">
@@ -1708,10 +1708,10 @@
         <v>40756</v>
       </c>
       <c r="B117" t="n">
-        <v>0.06489778610713119</v>
+        <v>0.06484968310646648</v>
       </c>
       <c r="C117" t="n">
-        <v>0.05390907951500711</v>
+        <v>0.05405938994113409</v>
       </c>
     </row>
     <row r="118">
@@ -1719,10 +1719,10 @@
         <v>40787</v>
       </c>
       <c r="B118" t="n">
-        <v>0.06357307830740264</v>
+        <v>0.06349977574657696</v>
       </c>
       <c r="C118" t="n">
-        <v>0.05263321385613327</v>
+        <v>0.05280210599504204</v>
       </c>
     </row>
     <row r="119">
@@ -1730,10 +1730,10 @@
         <v>40817</v>
       </c>
       <c r="B119" t="n">
-        <v>0.06451231820757986</v>
+        <v>0.06437173389605315</v>
       </c>
       <c r="C119" t="n">
-        <v>0.05348971824036437</v>
+        <v>0.053609598077621</v>
       </c>
     </row>
     <row r="120">
@@ -1741,10 +1741,10 @@
         <v>40848</v>
       </c>
       <c r="B120" t="n">
-        <v>0.06413490617156041</v>
+        <v>0.06421994265950433</v>
       </c>
       <c r="C120" t="n">
-        <v>0.05310408265549638</v>
+        <v>0.05329849656603667</v>
       </c>
     </row>
     <row r="121">
@@ -1752,10 +1752,10 @@
         <v>40878</v>
       </c>
       <c r="B121" t="n">
-        <v>0.06563416581082608</v>
+        <v>0.06577214645156663</v>
       </c>
       <c r="C121" t="n">
-        <v>0.05419032422790254</v>
+        <v>0.05432240592379507</v>
       </c>
     </row>
     <row r="122">
@@ -1774,10 +1774,10 @@
         <v>40940</v>
       </c>
       <c r="B123" t="n">
-        <v>0.06493000319669796</v>
+        <v>0.06523215775566363</v>
       </c>
       <c r="C123" t="n">
-        <v>0.05323671616582334</v>
+        <v>0.05342594939748113</v>
       </c>
     </row>
     <row r="124">
@@ -1785,10 +1785,10 @@
         <v>40969</v>
       </c>
       <c r="B124" t="n">
-        <v>0.06445562181086931</v>
+        <v>0.06513369674334035</v>
       </c>
       <c r="C124" t="n">
-        <v>0.05288806991599729</v>
+        <v>0.0535254957326818</v>
       </c>
     </row>
     <row r="125">
@@ -1796,10 +1796,10 @@
         <v>41000</v>
       </c>
       <c r="B125" t="n">
-        <v>0.06671489558546491</v>
+        <v>0.06733056239229844</v>
       </c>
       <c r="C125" t="n">
-        <v>0.05493202265349707</v>
+        <v>0.05551970234358968</v>
       </c>
     </row>
     <row r="126">
@@ -1807,10 +1807,10 @@
         <v>41030</v>
       </c>
       <c r="B126" t="n">
-        <v>0.06652349518817537</v>
+        <v>0.06702262977319697</v>
       </c>
       <c r="C126" t="n">
-        <v>0.05459808824382724</v>
+        <v>0.0551319790005243</v>
       </c>
     </row>
     <row r="127">
@@ -1818,10 +1818,10 @@
         <v>41061</v>
       </c>
       <c r="B127" t="n">
-        <v>0.06771129048579282</v>
+        <v>0.06812852725738217</v>
       </c>
       <c r="C127" t="n">
-        <v>0.05557175457036927</v>
+        <v>0.05606812008451902</v>
       </c>
     </row>
     <row r="128">
@@ -1829,10 +1829,10 @@
         <v>41091</v>
       </c>
       <c r="B128" t="n">
-        <v>0.06822045091599549</v>
+        <v>0.06840957232944141</v>
       </c>
       <c r="C128" t="n">
-        <v>0.05570758409431516</v>
+        <v>0.05606470017822106</v>
       </c>
     </row>
     <row r="129">
@@ -1840,10 +1840,10 @@
         <v>41122</v>
       </c>
       <c r="B129" t="n">
-        <v>0.07069760081377409</v>
+        <v>0.07064949781310938</v>
       </c>
       <c r="C129" t="n">
-        <v>0.05726989471269293</v>
+        <v>0.05742020513881991</v>
       </c>
     </row>
     <row r="130">
@@ -1851,10 +1851,10 @@
         <v>41153</v>
       </c>
       <c r="B130" t="n">
-        <v>0.07099281834136614</v>
+        <v>0.07091951578054047</v>
       </c>
       <c r="C130" t="n">
-        <v>0.05789474063285222</v>
+        <v>0.05806363277176099</v>
       </c>
     </row>
     <row r="131">
@@ -1862,10 +1862,10 @@
         <v>41183</v>
       </c>
       <c r="B131" t="n">
-        <v>0.07172429045612402</v>
+        <v>0.07158370614459732</v>
       </c>
       <c r="C131" t="n">
-        <v>0.05845315456943313</v>
+        <v>0.05857303440668976</v>
       </c>
     </row>
     <row r="132">
@@ -1873,10 +1873,10 @@
         <v>41214</v>
       </c>
       <c r="B132" t="n">
-        <v>0.07303950149215742</v>
+        <v>0.07312453798010134</v>
       </c>
       <c r="C132" t="n">
-        <v>0.05945777296124336</v>
+        <v>0.05965218687178366</v>
       </c>
     </row>
     <row r="133">
@@ -1884,10 +1884,10 @@
         <v>41244</v>
       </c>
       <c r="B133" t="n">
-        <v>0.06843829242972985</v>
+        <v>0.06857627307047041</v>
       </c>
       <c r="C133" t="n">
-        <v>0.05613796011551613</v>
+        <v>0.05627004181140866</v>
       </c>
     </row>
     <row r="134">
@@ -1906,10 +1906,10 @@
         <v>41306</v>
       </c>
       <c r="B135" t="n">
-        <v>0.07094049122352794</v>
+        <v>0.0712426457824936</v>
       </c>
       <c r="C135" t="n">
-        <v>0.0570390848052859</v>
+        <v>0.05722831803694368</v>
       </c>
     </row>
     <row r="136">
@@ -1917,10 +1917,10 @@
         <v>41334</v>
       </c>
       <c r="B136" t="n">
-        <v>0.07142240052599071</v>
+        <v>0.07210047545846175</v>
       </c>
       <c r="C136" t="n">
-        <v>0.05767958392977417</v>
+        <v>0.05831700974645869</v>
       </c>
     </row>
     <row r="137">
@@ -1928,10 +1928,10 @@
         <v>41365</v>
       </c>
       <c r="B137" t="n">
-        <v>0.07257981091089118</v>
+        <v>0.07319547771772471</v>
       </c>
       <c r="C137" t="n">
-        <v>0.05744489986289433</v>
+        <v>0.05803257955298693</v>
       </c>
     </row>
     <row r="138">
@@ -1939,10 +1939,10 @@
         <v>41395</v>
       </c>
       <c r="B138" t="n">
-        <v>0.07356671662847793</v>
+        <v>0.07406585121349953</v>
       </c>
       <c r="C138" t="n">
-        <v>0.05807947087940016</v>
+        <v>0.05861336163609722</v>
       </c>
     </row>
     <row r="139">
@@ -1950,10 +1950,10 @@
         <v>41426</v>
       </c>
       <c r="B139" t="n">
-        <v>0.0718011453867954</v>
+        <v>0.07221838215838475</v>
       </c>
       <c r="C139" t="n">
-        <v>0.0567200173248367</v>
+        <v>0.05721638283898645</v>
       </c>
     </row>
     <row r="140">
@@ -1961,10 +1961,10 @@
         <v>41456</v>
       </c>
       <c r="B140" t="n">
-        <v>0.07529805919304908</v>
+        <v>0.07548718060649499</v>
       </c>
       <c r="C140" t="n">
-        <v>0.05949410480395907</v>
+        <v>0.05985122088786497</v>
       </c>
     </row>
     <row r="141">
@@ -1972,10 +1972,10 @@
         <v>41487</v>
       </c>
       <c r="B141" t="n">
-        <v>0.07921145501673688</v>
+        <v>0.07916335201607216</v>
       </c>
       <c r="C141" t="n">
-        <v>0.06217414218893507</v>
+        <v>0.06232445261506205</v>
       </c>
     </row>
     <row r="142">
@@ -1983,10 +1983,10 @@
         <v>41518</v>
       </c>
       <c r="B142" t="n">
-        <v>0.08069707597439035</v>
+        <v>0.08062377341356468</v>
       </c>
       <c r="C142" t="n">
-        <v>0.06312320551732013</v>
+        <v>0.06329209765622891</v>
       </c>
     </row>
     <row r="143">
@@ -1994,10 +1994,10 @@
         <v>41548</v>
       </c>
       <c r="B143" t="n">
-        <v>0.08058729292843181</v>
+        <v>0.0804467086169051</v>
       </c>
       <c r="C143" t="n">
-        <v>0.06332201950979714</v>
+        <v>0.06344189934705378</v>
       </c>
     </row>
     <row r="144">
@@ -2005,10 +2005,10 @@
         <v>41579</v>
       </c>
       <c r="B144" t="n">
-        <v>0.07569660659203899</v>
+        <v>0.0757816430799829</v>
       </c>
       <c r="C144" t="n">
-        <v>0.05912179344370981</v>
+        <v>0.0593162073542501</v>
       </c>
     </row>
     <row r="145">
@@ -2016,10 +2016,10 @@
         <v>41609</v>
       </c>
       <c r="B145" t="n">
-        <v>0.07762776106124759</v>
+        <v>0.07776574170198815</v>
       </c>
       <c r="C145" t="n">
-        <v>0.06080820888989803</v>
+        <v>0.06094029058579056</v>
       </c>
     </row>
     <row r="146">
@@ -2038,10 +2038,10 @@
         <v>41671</v>
       </c>
       <c r="B147" t="n">
-        <v>0.07927684060414059</v>
+        <v>0.07957899516310625</v>
       </c>
       <c r="C147" t="n">
-        <v>0.06199064462257037</v>
+        <v>0.06217987785422815</v>
       </c>
     </row>
     <row r="148">
@@ -2049,10 +2049,10 @@
         <v>41699</v>
       </c>
       <c r="B148" t="n">
-        <v>0.0796424776996833</v>
+        <v>0.08032055263215435</v>
       </c>
       <c r="C148" t="n">
-        <v>0.06253190978293421</v>
+        <v>0.06316933559961874</v>
       </c>
     </row>
     <row r="149">
@@ -2060,10 +2060,10 @@
         <v>41730</v>
       </c>
       <c r="B149" t="n">
-        <v>0.08174743036503518</v>
+        <v>0.08236309717186871</v>
       </c>
       <c r="C149" t="n">
-        <v>0.06410226986939764</v>
+        <v>0.06468994955949026</v>
       </c>
     </row>
     <row r="150">
@@ -2071,10 +2071,10 @@
         <v>41760</v>
       </c>
       <c r="B150" t="n">
-        <v>0.08454666862638671</v>
+        <v>0.08504580321140831</v>
       </c>
       <c r="C150" t="n">
-        <v>0.06625078982309481</v>
+        <v>0.06678468057979187</v>
       </c>
     </row>
     <row r="151">
@@ -2082,10 +2082,10 @@
         <v>41791</v>
       </c>
       <c r="B151" t="n">
-        <v>0.08249935206916065</v>
+        <v>0.08291658884075</v>
       </c>
       <c r="C151" t="n">
-        <v>0.0649975148517372</v>
+        <v>0.06549388036588695</v>
       </c>
     </row>
     <row r="152">
@@ -2093,10 +2093,10 @@
         <v>41821</v>
       </c>
       <c r="B152" t="n">
-        <v>0.08466981657146383</v>
+        <v>0.08485893798490975</v>
       </c>
       <c r="C152" t="n">
-        <v>0.06616938206140469</v>
+        <v>0.0665264981453106</v>
       </c>
     </row>
     <row r="153">
@@ -2104,10 +2104,10 @@
         <v>41852</v>
       </c>
       <c r="B153" t="n">
-        <v>0.08624951807675565</v>
+        <v>0.08620141507609094</v>
       </c>
       <c r="C153" t="n">
-        <v>0.06711512666371414</v>
+        <v>0.06726543708984112</v>
       </c>
     </row>
     <row r="154">
@@ -2115,10 +2115,10 @@
         <v>41883</v>
       </c>
       <c r="B154" t="n">
-        <v>0.08500396800446541</v>
+        <v>0.08493066544363974</v>
       </c>
       <c r="C154" t="n">
-        <v>0.06642991787766095</v>
+        <v>0.06659881001656973</v>
       </c>
     </row>
     <row r="155">
@@ -2126,10 +2126,10 @@
         <v>41913</v>
       </c>
       <c r="B155" t="n">
-        <v>0.08475904770035679</v>
+        <v>0.08461846338883008</v>
       </c>
       <c r="C155" t="n">
-        <v>0.06553304949668515</v>
+        <v>0.06565292933394179</v>
       </c>
     </row>
     <row r="156">
@@ -2137,10 +2137,10 @@
         <v>41944</v>
       </c>
       <c r="B156" t="n">
-        <v>0.08627122729564218</v>
+        <v>0.0863562637835861</v>
       </c>
       <c r="C156" t="n">
-        <v>0.06676514060773553</v>
+        <v>0.06695955451827582</v>
       </c>
     </row>
     <row r="157">
@@ -2148,10 +2148,10 @@
         <v>41974</v>
       </c>
       <c r="B157" t="n">
-        <v>0.07955948734483023</v>
+        <v>0.07969746798557079</v>
       </c>
       <c r="C157" t="n">
-        <v>0.06179864419549007</v>
+        <v>0.06193072589138259</v>
       </c>
     </row>
     <row r="158">
@@ -2170,10 +2170,10 @@
         <v>42036</v>
       </c>
       <c r="B159" t="n">
-        <v>0.07640503997612043</v>
+        <v>0.07670719453508609</v>
       </c>
       <c r="C159" t="n">
-        <v>0.06025189274767184</v>
+        <v>0.06044112597932963</v>
       </c>
     </row>
     <row r="160">
@@ -2181,10 +2181,10 @@
         <v>42064</v>
       </c>
       <c r="B160" t="n">
-        <v>0.07647113172869466</v>
+        <v>0.0771492066611657</v>
       </c>
       <c r="C160" t="n">
-        <v>0.06047244617106159</v>
+        <v>0.0611098719877461</v>
       </c>
     </row>
     <row r="161">
@@ -2192,10 +2192,10 @@
         <v>42095</v>
       </c>
       <c r="B161" t="n">
-        <v>0.07654173988605513</v>
+        <v>0.07715740669288866</v>
       </c>
       <c r="C161" t="n">
-        <v>0.06098882887208067</v>
+        <v>0.06157650856217328</v>
       </c>
     </row>
     <row r="162">
@@ -2203,10 +2203,10 @@
         <v>42125</v>
       </c>
       <c r="B162" t="n">
-        <v>0.07895840873377283</v>
+        <v>0.07945754331879443</v>
       </c>
       <c r="C162" t="n">
-        <v>0.06267838879097574</v>
+        <v>0.06321227954767281</v>
       </c>
     </row>
     <row r="163">
@@ -2214,10 +2214,10 @@
         <v>42156</v>
       </c>
       <c r="B163" t="n">
-        <v>0.07730977436770553</v>
+        <v>0.07772701113929488</v>
       </c>
       <c r="C163" t="n">
-        <v>0.06228974898553095</v>
+        <v>0.0627861144996807</v>
       </c>
     </row>
     <row r="164">
@@ -2225,10 +2225,10 @@
         <v>42186</v>
       </c>
       <c r="B164" t="n">
-        <v>0.0733632133842918</v>
+        <v>0.07355233479773772</v>
       </c>
       <c r="C164" t="n">
-        <v>0.06034880596489933</v>
+        <v>0.06070592204880524</v>
       </c>
     </row>
     <row r="165">
@@ -2236,10 +2236,10 @@
         <v>42217</v>
       </c>
       <c r="B165" t="n">
-        <v>0.07529711020433942</v>
+        <v>0.07524900720367471</v>
       </c>
       <c r="C165" t="n">
-        <v>0.06207646868734846</v>
+        <v>0.06222677911347544</v>
       </c>
     </row>
     <row r="166">
@@ -2247,10 +2247,10 @@
         <v>42248</v>
       </c>
       <c r="B166" t="n">
-        <v>0.07645222971093295</v>
+        <v>0.07637892715010727</v>
       </c>
       <c r="C166" t="n">
-        <v>0.06275832907042664</v>
+        <v>0.06292722120933542</v>
       </c>
     </row>
     <row r="167">
@@ -2258,10 +2258,10 @@
         <v>42278</v>
       </c>
       <c r="B167" t="n">
-        <v>0.07713724354642033</v>
+        <v>0.07699665923489363</v>
       </c>
       <c r="C167" t="n">
-        <v>0.06324756371123129</v>
+        <v>0.06336744354848793</v>
       </c>
     </row>
     <row r="168">
@@ -2269,10 +2269,10 @@
         <v>42309</v>
       </c>
       <c r="B168" t="n">
-        <v>0.0799993613002858</v>
+        <v>0.08008439778822972</v>
       </c>
       <c r="C168" t="n">
-        <v>0.06513604151813676</v>
+        <v>0.06533045542867705</v>
       </c>
     </row>
     <row r="169">
@@ -2280,10 +2280,10 @@
         <v>42339</v>
       </c>
       <c r="B169" t="n">
-        <v>0.07686998521764705</v>
+        <v>0.07700796585838761</v>
       </c>
       <c r="C169" t="n">
-        <v>0.0631159612954327</v>
+        <v>0.06324804299132522</v>
       </c>
     </row>
     <row r="170">
@@ -2302,10 +2302,10 @@
         <v>42401</v>
       </c>
       <c r="B171" t="n">
-        <v>0.07501074957885372</v>
+        <v>0.07531290413781938</v>
       </c>
       <c r="C171" t="n">
-        <v>0.06188718218339316</v>
+        <v>0.06207641541505095</v>
       </c>
     </row>
     <row r="172">
@@ -2313,10 +2313,10 @@
         <v>42430</v>
       </c>
       <c r="B172" t="n">
-        <v>0.07467420477143448</v>
+        <v>0.07535227970390553</v>
       </c>
       <c r="C172" t="n">
-        <v>0.06186282585814736</v>
+        <v>0.06250025167483188</v>
       </c>
     </row>
     <row r="173">
@@ -2324,10 +2324,10 @@
         <v>42461</v>
       </c>
       <c r="B173" t="n">
-        <v>0.07413838658373612</v>
+        <v>0.07475405339056965</v>
       </c>
       <c r="C173" t="n">
-        <v>0.06141687045911193</v>
+        <v>0.06200455014920454</v>
       </c>
     </row>
     <row r="174">
@@ -2335,10 +2335,10 @@
         <v>42491</v>
       </c>
       <c r="B174" t="n">
-        <v>0.0740313783482623</v>
+        <v>0.0745305129332839</v>
       </c>
       <c r="C174" t="n">
-        <v>0.06323489829527788</v>
+        <v>0.06376878905197494</v>
       </c>
     </row>
     <row r="175">
@@ -2346,10 +2346,10 @@
         <v>42522</v>
       </c>
       <c r="B175" t="n">
-        <v>0.06756469391664523</v>
+        <v>0.06798193068823458</v>
       </c>
       <c r="C175" t="n">
-        <v>0.05784097747306542</v>
+        <v>0.05833734298721517</v>
       </c>
     </row>
     <row r="176">
@@ -2357,10 +2357,10 @@
         <v>42552</v>
       </c>
       <c r="B176" t="n">
-        <v>0.06967827324999983</v>
+        <v>0.06986739466344574</v>
       </c>
       <c r="C176" t="n">
-        <v>0.05950483477895994</v>
+        <v>0.05986195086286585</v>
       </c>
     </row>
     <row r="177">
@@ -2368,10 +2368,10 @@
         <v>42583</v>
       </c>
       <c r="B177" t="n">
-        <v>0.06863499732264003</v>
+        <v>0.06858689432197532</v>
       </c>
       <c r="C177" t="n">
-        <v>0.05893964999039447</v>
+        <v>0.05908996041652145</v>
       </c>
     </row>
     <row r="178">
@@ -2379,10 +2379,10 @@
         <v>42614</v>
       </c>
       <c r="B178" t="n">
-        <v>0.06851255074819368</v>
+        <v>0.068439248187368</v>
       </c>
       <c r="C178" t="n">
-        <v>0.0587477083123134</v>
+        <v>0.05891660045122218</v>
       </c>
     </row>
     <row r="179">
@@ -2390,10 +2390,10 @@
         <v>42644</v>
       </c>
       <c r="B179" t="n">
-        <v>0.06919025922658853</v>
+        <v>0.06904967491506182</v>
       </c>
       <c r="C179" t="n">
-        <v>0.05869453067163501</v>
+        <v>0.05881441050889165</v>
       </c>
     </row>
     <row r="180">
@@ -2401,10 +2401,10 @@
         <v>42675</v>
       </c>
       <c r="B180" t="n">
-        <v>0.07043846617566533</v>
+        <v>0.07052350266360925</v>
       </c>
       <c r="C180" t="n">
-        <v>0.0594497131741213</v>
+        <v>0.0596441270846616</v>
       </c>
     </row>
     <row r="181">
@@ -2412,10 +2412,10 @@
         <v>42705</v>
       </c>
       <c r="B181" t="n">
-        <v>0.06868365971916049</v>
+        <v>0.06882164035990104</v>
       </c>
       <c r="C181" t="n">
-        <v>0.05790713873302084</v>
+        <v>0.05803922042891337</v>
       </c>
     </row>
     <row r="182">
@@ -2434,10 +2434,10 @@
         <v>42767</v>
       </c>
       <c r="B183" t="n">
-        <v>0.06671581620910168</v>
+        <v>0.06701797076806734</v>
       </c>
       <c r="C183" t="n">
-        <v>0.05694613981251462</v>
+        <v>0.05713537304417241</v>
       </c>
     </row>
     <row r="184">
@@ -2445,10 +2445,10 @@
         <v>42795</v>
       </c>
       <c r="B184" t="n">
-        <v>0.06484069589671997</v>
+        <v>0.06551877082919101</v>
       </c>
       <c r="C184" t="n">
-        <v>0.05458885075838964</v>
+        <v>0.05522627657507416</v>
       </c>
     </row>
     <row r="185">
@@ -2456,10 +2456,10 @@
         <v>42826</v>
       </c>
       <c r="B185" t="n">
-        <v>0.06552059772474558</v>
+        <v>0.06613626453157911</v>
       </c>
       <c r="C185" t="n">
-        <v>0.0550380112645453</v>
+        <v>0.05562569095463791</v>
       </c>
     </row>
     <row r="186">
@@ -2467,10 +2467,10 @@
         <v>42856</v>
       </c>
       <c r="B186" t="n">
-        <v>0.0647764296481842</v>
+        <v>0.0652755642332058</v>
       </c>
       <c r="C186" t="n">
-        <v>0.05462680988041402</v>
+        <v>0.05516070063711108</v>
       </c>
     </row>
     <row r="187">
@@ -2478,10 +2478,10 @@
         <v>42887</v>
       </c>
       <c r="B187" t="n">
-        <v>0.06518829495856299</v>
+        <v>0.06560553173015234</v>
       </c>
       <c r="C187" t="n">
-        <v>0.05478857969685992</v>
+        <v>0.05528494521100967</v>
       </c>
     </row>
     <row r="188">
@@ -2489,10 +2489,10 @@
         <v>42917</v>
       </c>
       <c r="B188" t="n">
-        <v>0.06545336722166187</v>
+        <v>0.06564248863510778</v>
       </c>
       <c r="C188" t="n">
-        <v>0.054934086496212</v>
+        <v>0.0552912025801179</v>
       </c>
     </row>
     <row r="189">
@@ -2500,10 +2500,10 @@
         <v>42948</v>
       </c>
       <c r="B189" t="n">
-        <v>0.06593444637181607</v>
+        <v>0.06588634337115136</v>
       </c>
       <c r="C189" t="n">
-        <v>0.055067736475134</v>
+        <v>0.05521804690126098</v>
       </c>
     </row>
     <row r="190">
@@ -2511,10 +2511,10 @@
         <v>42979</v>
       </c>
       <c r="B190" t="n">
-        <v>0.06624710538407418</v>
+        <v>0.0661738028232485</v>
       </c>
       <c r="C190" t="n">
-        <v>0.05534823504469731</v>
+        <v>0.05551712718360609</v>
       </c>
     </row>
     <row r="191">
@@ -2522,10 +2522,10 @@
         <v>43009</v>
       </c>
       <c r="B191" t="n">
-        <v>0.06825558734679694</v>
+        <v>0.06811500303527024</v>
       </c>
       <c r="C191" t="n">
-        <v>0.05730779334311174</v>
+        <v>0.05742767318036837</v>
       </c>
     </row>
     <row r="192">
@@ -2533,10 +2533,10 @@
         <v>43040</v>
       </c>
       <c r="B192" t="n">
-        <v>0.06927933086674376</v>
+        <v>0.06936436735468768</v>
       </c>
       <c r="C192" t="n">
-        <v>0.05794813674218686</v>
+        <v>0.05814255065272716</v>
       </c>
     </row>
     <row r="193">
@@ -2544,10 +2544,10 @@
         <v>43070</v>
       </c>
       <c r="B193" t="n">
-        <v>0.07026732777374455</v>
+        <v>0.0704053084144851</v>
       </c>
       <c r="C193" t="n">
-        <v>0.05877354044944504</v>
+        <v>0.05890562214533756</v>
       </c>
     </row>
     <row r="194">
@@ -2566,10 +2566,10 @@
         <v>43132</v>
       </c>
       <c r="B195" t="n">
-        <v>0.07054913001473033</v>
+        <v>0.07085128457369599</v>
       </c>
       <c r="C195" t="n">
-        <v>0.05871728864863272</v>
+        <v>0.0589065218802905</v>
       </c>
     </row>
     <row r="196">
@@ -2577,10 +2577,10 @@
         <v>43160</v>
       </c>
       <c r="B196" t="n">
-        <v>0.07190904141660984</v>
+        <v>0.07258711634908088</v>
       </c>
       <c r="C196" t="n">
-        <v>0.06058360528491092</v>
+        <v>0.06122103110159544</v>
       </c>
     </row>
     <row r="197">
@@ -2588,10 +2588,10 @@
         <v>43191</v>
       </c>
       <c r="B197" t="n">
-        <v>0.07202639372734224</v>
+        <v>0.07264206053417577</v>
       </c>
       <c r="C197" t="n">
-        <v>0.06105741813597244</v>
+        <v>0.06164509782606505</v>
       </c>
     </row>
     <row r="198">
@@ -2599,10 +2599,10 @@
         <v>43221</v>
       </c>
       <c r="B198" t="n">
-        <v>0.07140728015031421</v>
+        <v>0.07190641473533581</v>
       </c>
       <c r="C198" t="n">
-        <v>0.05990217822633218</v>
+        <v>0.06043606898302924</v>
       </c>
     </row>
     <row r="199">
@@ -2610,10 +2610,10 @@
         <v>43252</v>
       </c>
       <c r="B199" t="n">
-        <v>0.07391909360696422</v>
+        <v>0.07433633037855357</v>
       </c>
       <c r="C199" t="n">
-        <v>0.0622927205961166</v>
+        <v>0.06278908611026635</v>
       </c>
     </row>
     <row r="200">
@@ -2621,10 +2621,10 @@
         <v>43282</v>
       </c>
       <c r="B200" t="n">
-        <v>0.07308869332032786</v>
+        <v>0.07327781473377377</v>
       </c>
       <c r="C200" t="n">
-        <v>0.06257882598397008</v>
+        <v>0.06293594206787599</v>
       </c>
     </row>
     <row r="201">
@@ -2632,10 +2632,10 @@
         <v>43313</v>
       </c>
       <c r="B201" t="n">
-        <v>0.0762970819686363</v>
+        <v>0.07624897896797159</v>
       </c>
       <c r="C201" t="n">
-        <v>0.06545169526619257</v>
+        <v>0.06560200569231955</v>
       </c>
     </row>
     <row r="202">
@@ -2643,10 +2643,10 @@
         <v>43344</v>
       </c>
       <c r="B202" t="n">
-        <v>0.07787530091916904</v>
+        <v>0.07780199835834337</v>
       </c>
       <c r="C202" t="n">
-        <v>0.06676280375430556</v>
+        <v>0.06693169589321434</v>
       </c>
     </row>
     <row r="203">
@@ -2654,10 +2654,10 @@
         <v>43374</v>
       </c>
       <c r="B203" t="n">
-        <v>0.0792748999987653</v>
+        <v>0.0791343156872386</v>
       </c>
       <c r="C203" t="n">
-        <v>0.06822945181799106</v>
+        <v>0.0683493316552477</v>
       </c>
     </row>
     <row r="204">
@@ -2665,10 +2665,10 @@
         <v>43405</v>
       </c>
       <c r="B204" t="n">
-        <v>0.07848626097795014</v>
+        <v>0.07857129746589406</v>
       </c>
       <c r="C204" t="n">
-        <v>0.06713651214476106</v>
+        <v>0.06733092605530135</v>
       </c>
     </row>
     <row r="205">
@@ -2676,10 +2676,10 @@
         <v>43435</v>
       </c>
       <c r="B205" t="n">
-        <v>0.08001520180010568</v>
+        <v>0.08015318244084624</v>
       </c>
       <c r="C205" t="n">
-        <v>0.06852537287031019</v>
+        <v>0.06865745456620272</v>
       </c>
     </row>
     <row r="206">
@@ -2698,10 +2698,10 @@
         <v>43497</v>
       </c>
       <c r="B207" t="n">
-        <v>0.07711822990169169</v>
+        <v>0.07742038446065735</v>
       </c>
       <c r="C207" t="n">
-        <v>0.06860465952547935</v>
+        <v>0.06879389275713714</v>
       </c>
     </row>
     <row r="208">
@@ -2709,10 +2709,10 @@
         <v>43525</v>
       </c>
       <c r="B208" t="n">
-        <v>0.07591849596560939</v>
+        <v>0.07659657089808043</v>
       </c>
       <c r="C208" t="n">
-        <v>0.06784819185275041</v>
+        <v>0.06848561766943494</v>
       </c>
     </row>
     <row r="209">
@@ -2720,10 +2720,10 @@
         <v>43556</v>
       </c>
       <c r="B209" t="n">
-        <v>0.07554332877341807</v>
+        <v>0.0761589955802516</v>
       </c>
       <c r="C209" t="n">
-        <v>0.06834608810663377</v>
+        <v>0.06893376779672639</v>
       </c>
     </row>
     <row r="210">
@@ -2731,10 +2731,10 @@
         <v>43586</v>
       </c>
       <c r="B210" t="n">
-        <v>0.0748671528348484</v>
+        <v>0.07536628741987</v>
       </c>
       <c r="C210" t="n">
-        <v>0.06708938421578131</v>
+        <v>0.06762327497247837</v>
       </c>
     </row>
     <row r="211">
@@ -2742,10 +2742,10 @@
         <v>43617</v>
       </c>
       <c r="B211" t="n">
-        <v>0.07518598095878748</v>
+        <v>0.07560321773037683</v>
       </c>
       <c r="C211" t="n">
-        <v>0.06597114047146146</v>
+        <v>0.06646750598561121</v>
       </c>
     </row>
     <row r="212">
@@ -2753,10 +2753,10 @@
         <v>43647</v>
       </c>
       <c r="B212" t="n">
-        <v>0.07666429178832071</v>
+        <v>0.07685341320176663</v>
       </c>
       <c r="C212" t="n">
-        <v>0.06728829996071789</v>
+        <v>0.0676454160446238</v>
       </c>
     </row>
     <row r="213">
@@ -2764,10 +2764,10 @@
         <v>43678</v>
       </c>
       <c r="B213" t="n">
-        <v>0.07691629649594268</v>
+        <v>0.07686819349527797</v>
       </c>
       <c r="C213" t="n">
-        <v>0.06814351463147256</v>
+        <v>0.06829382505759954</v>
       </c>
     </row>
     <row r="214">
@@ -2775,10 +2775,10 @@
         <v>43709</v>
       </c>
       <c r="B214" t="n">
-        <v>0.07695220471429706</v>
+        <v>0.07687890215347139</v>
       </c>
       <c r="C214" t="n">
-        <v>0.06818079350737592</v>
+        <v>0.0683496856462847</v>
       </c>
     </row>
     <row r="215">
@@ -2786,10 +2786,10 @@
         <v>43739</v>
       </c>
       <c r="B215" t="n">
-        <v>0.07735721110618074</v>
+        <v>0.07721662679465403</v>
       </c>
       <c r="C215" t="n">
-        <v>0.06861447636249061</v>
+        <v>0.06873435619974726</v>
       </c>
     </row>
     <row r="216">
@@ -2797,10 +2797,10 @@
         <v>43770</v>
       </c>
       <c r="B216" t="n">
-        <v>0.07951360287008191</v>
+        <v>0.07959863935802583</v>
       </c>
       <c r="C216" t="n">
-        <v>0.07008687691708422</v>
+        <v>0.07028129082762451</v>
       </c>
     </row>
     <row r="217">
@@ -2808,10 +2808,10 @@
         <v>43800</v>
       </c>
       <c r="B217" t="n">
-        <v>0.08097226192064176</v>
+        <v>0.08111024256138231</v>
       </c>
       <c r="C217" t="n">
-        <v>0.07236509152765577</v>
+        <v>0.0724971732235483</v>
       </c>
     </row>
     <row r="218">
@@ -2830,384 +2830,10 @@
         <v>43862</v>
       </c>
       <c r="B219" t="n">
-        <v>0.07745365246448951</v>
+        <v>0.07775580702345518</v>
       </c>
       <c r="C219" t="n">
-        <v>0.06941479951770366</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" s="1" t="n">
-        <v>43891</v>
-      </c>
-      <c r="B220" t="n">
-        <v>0.07640591717700999</v>
-      </c>
-      <c r="C220" t="n">
-        <v>0.06974404093594504</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" s="1" t="n">
-        <v>43922</v>
-      </c>
-      <c r="B221" t="n">
-        <v>0.07541543745729969</v>
-      </c>
-      <c r="C221" t="n">
-        <v>0.06847120647983108</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" s="1" t="n">
-        <v>43952</v>
-      </c>
-      <c r="B222" t="n">
-        <v>0.07435209886669174</v>
-      </c>
-      <c r="C222" t="n">
-        <v>0.06760851439750712</v>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" s="1" t="n">
-        <v>43983</v>
-      </c>
-      <c r="B223" t="n">
-        <v>0.07426830870131311</v>
-      </c>
-      <c r="C223" t="n">
-        <v>0.0682227680156024</v>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" s="1" t="n">
-        <v>44013</v>
-      </c>
-      <c r="B224" t="n">
-        <v>0.06655340346522796</v>
-      </c>
-      <c r="C224" t="n">
-        <v>0.06291930812048031</v>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" s="1" t="n">
-        <v>44044</v>
-      </c>
-      <c r="B225" t="n">
-        <v>0.06276609378786076</v>
-      </c>
-      <c r="C225" t="n">
-        <v>0.0600026305235625</v>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" s="1" t="n">
-        <v>44075</v>
-      </c>
-      <c r="B226" t="n">
-        <v>0.06017986948882903</v>
-      </c>
-      <c r="C226" t="n">
-        <v>0.05864331103308755</v>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" s="1" t="n">
-        <v>44105</v>
-      </c>
-      <c r="B227" t="n">
-        <v>0.05573083719191907</v>
-      </c>
-      <c r="C227" t="n">
-        <v>0.05547551112428134</v>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" s="1" t="n">
-        <v>44136</v>
-      </c>
-      <c r="B228" t="n">
-        <v>0.0552284635438467</v>
-      </c>
-      <c r="C228" t="n">
-        <v>0.05464692351543116</v>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" s="1" t="n">
-        <v>44166</v>
-      </c>
-      <c r="B229" t="n">
-        <v>0.05581111897776039</v>
-      </c>
-      <c r="C229" t="n">
-        <v>0.05485666932588031</v>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" s="1" t="n">
-        <v>44197</v>
-      </c>
-      <c r="B230" t="n">
-        <v>0.05140672522087975</v>
-      </c>
-      <c r="C230" t="n">
-        <v>0.050776876665728</v>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" s="1" t="n">
-        <v>44228</v>
-      </c>
-      <c r="B231" t="n">
-        <v>0.05651519511058319</v>
-      </c>
-      <c r="C231" t="n">
-        <v>0.05386078602591986</v>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" s="1" t="n">
-        <v>44256</v>
-      </c>
-      <c r="B232" t="n">
-        <v>0.06127206726587887</v>
-      </c>
-      <c r="C232" t="n">
-        <v>0.05662933764893108</v>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" s="1" t="n">
-        <v>44287</v>
-      </c>
-      <c r="B233" t="n">
-        <v>0.06199990692898107</v>
-      </c>
-      <c r="C233" t="n">
-        <v>0.05750522911676381</v>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" s="1" t="n">
-        <v>44317</v>
-      </c>
-      <c r="B234" t="n">
-        <v>0.0623416157031278</v>
-      </c>
-      <c r="C234" t="n">
-        <v>0.05844169728161413</v>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" s="1" t="n">
-        <v>44348</v>
-      </c>
-      <c r="B235" t="n">
-        <v>0.05975238687748505</v>
-      </c>
-      <c r="C235" t="n">
-        <v>0.05626074643955729</v>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" s="1" t="n">
-        <v>44378</v>
-      </c>
-      <c r="B236" t="n">
-        <v>0.06170993669510062</v>
-      </c>
-      <c r="C236" t="n">
-        <v>0.05784493374187512</v>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" s="1" t="n">
-        <v>44409</v>
-      </c>
-      <c r="B237" t="n">
-        <v>0.05988931461963712</v>
-      </c>
-      <c r="C237" t="n">
-        <v>0.05614597364977676</v>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" s="1" t="n">
-        <v>44440</v>
-      </c>
-      <c r="B238" t="n">
-        <v>0.0592030445096669</v>
-      </c>
-      <c r="C238" t="n">
-        <v>0.05607561073138858</v>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" s="1" t="n">
-        <v>44470</v>
-      </c>
-      <c r="B239" t="n">
-        <v>0.05952865034952588</v>
-      </c>
-      <c r="C239" t="n">
-        <v>0.05596146509360781</v>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" s="1" t="n">
-        <v>44501</v>
-      </c>
-      <c r="B240" t="n">
-        <v>0.06004569223128834</v>
-      </c>
-      <c r="C240" t="n">
-        <v>0.0559624340104178</v>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" s="1" t="n">
-        <v>44531</v>
-      </c>
-      <c r="B241" t="n">
-        <v>0.06021726288427684</v>
-      </c>
-      <c r="C241" t="n">
-        <v>0.05522388909170248</v>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" s="1" t="n">
-        <v>44562</v>
-      </c>
-      <c r="B242" t="n">
-        <v>0.0590542990322673</v>
-      </c>
-      <c r="C242" t="n">
-        <v>0.05389982758847553</v>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" s="1" t="n">
-        <v>44593</v>
-      </c>
-      <c r="B243" t="n">
-        <v>0.05891691680115835</v>
-      </c>
-      <c r="C243" t="n">
-        <v>0.05405791549026105</v>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" s="1" t="n">
-        <v>44621</v>
-      </c>
-      <c r="B244" t="n">
-        <v>0.05864183790975851</v>
-      </c>
-      <c r="C244" t="n">
-        <v>0.05397171032646551</v>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" s="1" t="n">
-        <v>44652</v>
-      </c>
-      <c r="B245" t="n">
-        <v>0.05706479400449736</v>
-      </c>
-      <c r="C245" t="n">
-        <v>0.05320409537187834</v>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" s="1" t="n">
-        <v>44682</v>
-      </c>
-      <c r="B246" t="n">
-        <v>0.05497250612794705</v>
-      </c>
-      <c r="C246" t="n">
-        <v>0.05189299082401794</v>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" s="1" t="n">
-        <v>44713</v>
-      </c>
-      <c r="B247" t="n">
-        <v>0.05545502677679232</v>
-      </c>
-      <c r="C247" t="n">
-        <v>0.0525151060179146</v>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" s="1" t="n">
-        <v>44743</v>
-      </c>
-      <c r="B248" t="n">
-        <v>0.05638996804828432</v>
-      </c>
-      <c r="C248" t="n">
-        <v>0.05345876120211413</v>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" s="1" t="n">
-        <v>44774</v>
-      </c>
-      <c r="B249" t="n">
-        <v>0.05701152264672878</v>
-      </c>
-      <c r="C249" t="n">
-        <v>0.05408276938689588</v>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" s="1" t="n">
-        <v>44805</v>
-      </c>
-      <c r="B250" t="n">
-        <v>0.05911408727243805</v>
-      </c>
-      <c r="C250" t="n">
-        <v>0.05557779496161762</v>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" s="1" t="n">
-        <v>44835</v>
-      </c>
-      <c r="B251" t="n">
-        <v>0.06131010451647555</v>
-      </c>
-      <c r="C251" t="n">
-        <v>0.05770839141425196</v>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" s="1" t="n">
-        <v>44866</v>
-      </c>
-      <c r="B252" t="n">
-        <v>0.06464027297285999</v>
-      </c>
-      <c r="C252" t="n">
-        <v>0.05960849576118461</v>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" s="1" t="n">
-        <v>44896</v>
-      </c>
-      <c r="B253" t="n">
-        <v>0.06412270393590286</v>
-      </c>
-      <c r="C253" t="n">
-        <v>0.05874618734157668</v>
+        <v>0.06960403274936144</v>
       </c>
     </row>
   </sheetData>
@@ -3268,16 +2894,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.004348173296454249</v>
+        <v>0.003849038711432647</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.006026988576579212</v>
+        <v>-0.006164969217319771</v>
       </c>
       <c r="E2" t="n">
-        <v>0.01037516187303346</v>
+        <v>0.01001400792875242</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1119696776143911</v>
+        <v>0.2677850455608918</v>
       </c>
     </row>
     <row r="3">
@@ -3292,16 +2918,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.003019338245544285</v>
+        <v>0.002485447488847222</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.005304790008279665</v>
+        <v>-0.005436871704172187</v>
       </c>
       <c r="E3" t="n">
-        <v>0.008324128253823952</v>
+        <v>0.00792231919301941</v>
       </c>
       <c r="F3" t="n">
-        <v>0.4028763468778062</v>
+        <v>0.526575016434948</v>
       </c>
     </row>
   </sheetData>

</xml_diff>